<commit_message>
BinhLH_Update UI templates and project dependencies
- Added navBar and footer fragments to auth/reset-password.html
- Added footer fragment to booking/cancel-policy.html
- Updated pom.xml Spring Boot version and dependencies
- Fixed AutoConfigureMockMvc import in PageRenderSmokeTests.java
- Updated test data and reports (booking, wishlist)
- Added new banner image (Invicon_Emerald.png)
- Cleaned up temporary diff text files
</commit_message>
<xml_diff>
--- a/booking_test_data.xlsx
+++ b/booking_test_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\SE1912- Lop chuyen nganh\Offline\Ky_5\SWP391\project\hotel-management\SWP391_Group5_SU26_HotelsManagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7718D54A-F2B8-4DB7-B683-1A60BADEECE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{163787D0-E350-42A5-81F9-37BECA4213AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12468" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="35">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>customer_binh</t>
-  </si>
-  <si>
-    <t>123456</t>
   </si>
   <si>
     <t>Vinpearl Resort Nha Trang</t>
@@ -520,154 +517,154 @@
       <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2">
+        <v>12345678</v>
+      </c>
+      <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>13</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>15</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>16</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" t="s">
         <v>17</v>
-      </c>
-      <c r="I2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3">
+        <v>12345678</v>
+      </c>
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>15</v>
       </c>
-      <c r="G3" t="s">
-        <v>16</v>
-      </c>
       <c r="H3" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" t="s">
         <v>20</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>21</v>
-      </c>
-      <c r="J3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4">
+        <v>12345678</v>
+      </c>
+      <c r="D4" t="s">
         <v>12</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>13</v>
       </c>
-      <c r="E4" t="s">
-        <v>14</v>
-      </c>
       <c r="G4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" t="s">
         <v>24</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>25</v>
-      </c>
-      <c r="J4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
         <v>27</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5">
+        <v>12345678</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
         <v>28</v>
       </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>29</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>30</v>
-      </c>
-      <c r="J5" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6">
+        <v>12345678</v>
+      </c>
+      <c r="D6" t="s">
         <v>12</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>13</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>14</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>15</v>
       </c>
-      <c r="G6" t="s">
-        <v>16</v>
-      </c>
       <c r="H6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" t="s">
         <v>33</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>34</v>
-      </c>
-      <c r="J6" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>